<commit_message>
Update with August 26 presentations
Update with August 26 presentations
</commit_message>
<xml_diff>
--- a/3_Scholarly_Activity/3_0_Misc/research_activity.xlsx
+++ b/3_Scholarly_Activity/3_0_Misc/research_activity.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dcham\Documents\GitHub\Chamberlain_Tenure_Packet\3_Scholarly_Activity\3_0_Misc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chambd17\Documents\GitHub\Chamberlain_Tenure_Packet\3_Scholarly_Activity\3_0_Misc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B315D67-D0BD-4E07-9540-0A8877F7925B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6D95B89-C410-49DF-8F0B-6054E7BEB1B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1305" yWindow="2430" windowWidth="16755" windowHeight="17655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="activity" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">activity!$A$1:$F$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">activity!$A$1:$F$46</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="82">
   <si>
     <t>Type</t>
   </si>
@@ -352,6 +352,23 @@
     <t>Dux Speltz, E.*, Chamberlain Jr., D., Aik, M., Blood, B., &amp; Zaldivar, Z. (2026, June 2). From
 expert habits to student support: Using process-tracing tools to build process-focused GenAI writing
 guidance. SIG Writing Conference, Winterthur, Switzerland.</t>
+  </si>
+  <si>
+    <t>26-27</t>
+  </si>
+  <si>
+    <t>Chamberlain Jr., D.*, Jeter, R., &amp; Rozier, K. (2026, Aug 5-8). Identifying Qualitative Features of Mathematics Assessment Items for Validity and Reliability. Mathematical Association of America
+MathFest, Boston, MA.</t>
+  </si>
+  <si>
+    <t>Jeter, R.*, Chamberlain Jr., D., &amp; Rozier, K. (2026, Aug 5-8). Discovering Latent Structure in
+Low-Stakes Calculus Assessments via Unsupervised Learning. Mathematical Association of America
+MathFest, Boston, MA.</t>
+  </si>
+  <si>
+    <t>Stell, T.*, Jeter, R., Chamberlain Jr., D., &amp; Rozier, K. (2026, Aug 5-8). The Distractor Dilemma:
+Shortcomings of LLMs in Diagnosing Specific Algebraic Misconceptions. Mathematical Association
+of America MathFest, Boston, MA.</t>
   </si>
 </sst>
 </file>
@@ -670,17 +687,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:F46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F49"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -696,11 +712,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -720,7 +736,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -740,7 +756,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -760,7 +776,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -780,7 +796,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -800,7 +816,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -820,7 +836,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -840,7 +856,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -860,7 +876,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -880,7 +896,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -900,7 +916,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -920,7 +936,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>6</v>
       </c>
@@ -940,7 +956,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>6</v>
       </c>
@@ -960,7 +976,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>6</v>
       </c>
@@ -980,7 +996,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -996,11 +1012,11 @@
       <c r="E16" t="s">
         <v>9</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="F16" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -1016,11 +1032,11 @@
       <c r="E17" t="s">
         <v>11</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F17" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -1036,11 +1052,11 @@
       <c r="E18" t="s">
         <v>33</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -1056,11 +1072,11 @@
       <c r="E19" t="s">
         <v>42</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -1076,11 +1092,11 @@
       <c r="E20" t="s">
         <v>33</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F20" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -1096,11 +1112,11 @@
       <c r="E21" t="s">
         <v>45</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="F21" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>36</v>
       </c>
@@ -1116,11 +1132,11 @@
       <c r="E22" t="s">
         <v>32</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="F22" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1136,11 +1152,11 @@
       <c r="E23" t="s">
         <v>42</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="F23" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>36</v>
       </c>
@@ -1156,11 +1172,11 @@
       <c r="E24" t="s">
         <v>50</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="F24" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>36</v>
       </c>
@@ -1176,11 +1192,11 @@
       <c r="E25" t="s">
         <v>42</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F25" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>36</v>
       </c>
@@ -1196,11 +1212,11 @@
       <c r="E26" t="s">
         <v>9</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -1216,11 +1232,11 @@
       <c r="E27" t="s">
         <v>9</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F27" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>36</v>
       </c>
@@ -1236,11 +1252,11 @@
       <c r="E28" t="s">
         <v>9</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>36</v>
       </c>
@@ -1256,11 +1272,11 @@
       <c r="E29" t="s">
         <v>9</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="F29" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>36</v>
       </c>
@@ -1276,11 +1292,11 @@
       <c r="E30" t="s">
         <v>9</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="F30" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -1296,11 +1312,11 @@
       <c r="E31" t="s">
         <v>9</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="F31" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>58</v>
       </c>
@@ -1316,11 +1332,11 @@
       <c r="E32" t="s">
         <v>31</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="F32" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>58</v>
       </c>
@@ -1336,11 +1352,11 @@
       <c r="E33" t="s">
         <v>32</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="F33" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>58</v>
       </c>
@@ -1356,11 +1372,11 @@
       <c r="E34" t="s">
         <v>9</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="F34" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>58</v>
       </c>
@@ -1376,11 +1392,11 @@
       <c r="E35" t="s">
         <v>11</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="F35" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>58</v>
       </c>
@@ -1396,11 +1412,11 @@
       <c r="E36" t="s">
         <v>50</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="F36" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>58</v>
       </c>
@@ -1416,11 +1432,11 @@
       <c r="E37" t="s">
         <v>50</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="F37" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>58</v>
       </c>
@@ -1436,11 +1452,11 @@
       <c r="E38" t="s">
         <v>32</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="F38" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>58</v>
       </c>
@@ -1456,11 +1472,11 @@
       <c r="E39" t="s">
         <v>33</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="F39" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>58</v>
       </c>
@@ -1476,11 +1492,11 @@
       <c r="E40" t="s">
         <v>33</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="F40" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>58</v>
       </c>
@@ -1496,11 +1512,11 @@
       <c r="E41" t="s">
         <v>11</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="F41" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>58</v>
       </c>
@@ -1516,11 +1532,11 @@
       <c r="E42" t="s">
         <v>33</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="F42" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>58</v>
       </c>
@@ -1536,11 +1552,11 @@
       <c r="E43" t="s">
         <v>33</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="F43" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>58</v>
       </c>
@@ -1556,11 +1572,11 @@
       <c r="E44" t="s">
         <v>9</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="F44" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>58</v>
       </c>
@@ -1576,11 +1592,11 @@
       <c r="E45" t="s">
         <v>9</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="F45" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>58</v>
       </c>
@@ -1596,18 +1612,72 @@
       <c r="E46" t="s">
         <v>42</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F46" t="s">
         <v>77</v>
       </c>
     </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>58</v>
+      </c>
+      <c r="B47" t="s">
+        <v>59</v>
+      </c>
+      <c r="C47" t="s">
+        <v>78</v>
+      </c>
+      <c r="D47">
+        <v>2026</v>
+      </c>
+      <c r="E47" t="s">
+        <v>32</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>58</v>
+      </c>
+      <c r="B48" t="s">
+        <v>59</v>
+      </c>
+      <c r="C48" t="s">
+        <v>78</v>
+      </c>
+      <c r="D48">
+        <v>2026</v>
+      </c>
+      <c r="E48" t="s">
+        <v>32</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49" t="s">
+        <v>59</v>
+      </c>
+      <c r="C49" t="s">
+        <v>78</v>
+      </c>
+      <c r="D49">
+        <v>2026</v>
+      </c>
+      <c r="E49" t="s">
+        <v>32</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F45" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Presentation"/>
-        <filter val="Publication"/>
-      </filters>
-    </filterColumn>
+  <autoFilter ref="A1:F46" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F16">
       <sortCondition ref="C1:C16"/>
     </sortState>

</xml_diff>